<commit_message>
Document put strike risk tolerance
</commit_message>
<xml_diff>
--- a/models/builds/2026-07-31-Ganoza-eur-receivable-hedge-model.xlsx
+++ b/models/builds/2026-07-31-Ganoza-eur-receivable-hedge-model.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R44281085dc754e01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="2" r:id="Rf1af48dac28a4d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="R6dfe4483b55b449a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forwards" sheetId="4" r:id="R0913d2c21522401a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MoneyMarket" sheetId="5" r:id="Rc764f05d3b204e7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="6" r:id="R8c54163fe4e34a37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="Rf8200cc2dadd4200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="Rce92703c04f2427a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="9" r:id="Red89ae1f942744f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R105eb7a523f94048"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="2" r:id="R5c04a8d6939b4d11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="R1749a0d38b8448b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forwards" sheetId="4" r:id="R50ec3b6148a44d9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MoneyMarket" sheetId="5" r:id="Rd57ae1a20c0c4d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="6" r:id="Rc9af3cb5dfc440ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R34e836d2bf7c44b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R3ab1e7b326b34358"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="9" r:id="R99fbabb4d0514a9e"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="FC_AMT">'Inputs'!B2</x:definedName>
@@ -63,7 +63,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -90,6 +90,11 @@
         <x:fgColor rgb="FFD9D9D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -111,7 +116,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="46">
+  <x:cellXfs count="50">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -184,6 +189,14 @@
     <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -448,7 +461,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2f9cf387fa864280"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R17562561738f4e02"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1512,7 +1525,7 @@
     <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c77c425574445ad"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R311c4c59063d4bdc"/>
 </x:worksheet>
 </file>
 
@@ -1783,6 +1796,20 @@
         <x:v>Record tenor, strike, and premium</x:v>
       </x:c>
     </x:row>
+    <x:row r="12" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A12" s="49" t="str">
+        <x:v>Put strike risk tolerance</x:v>
+      </x:c>
+      <x:c r="B12" s="48" t="str">
+        <x:v>K_PUT = 1.00 protects a $4.41M net floor after premium</x:v>
+      </x:c>
+      <x:c r="C12" s="48" t="str">
+        <x:v>Decision required</x:v>
+      </x:c>
+      <x:c r="D12" s="48" t="str">
+        <x:v>This accepts a $0.10/EUR decline from spot before the floor binds; set the strike based on the USD floor the business requires.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
Populate EUR hedge model with Stage 4 market data
</commit_message>
<xml_diff>
--- a/models/builds/2026-07-31-Ganoza-eur-receivable-hedge-model.xlsx
+++ b/models/builds/2026-07-31-Ganoza-eur-receivable-hedge-model.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R105eb7a523f94048"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="2" r:id="R5c04a8d6939b4d11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="R1749a0d38b8448b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forwards" sheetId="4" r:id="R50ec3b6148a44d9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MoneyMarket" sheetId="5" r:id="Rd57ae1a20c0c4d6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="6" r:id="Rc9af3cb5dfc440ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R34e836d2bf7c44b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R3ab1e7b326b34358"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="9" r:id="R99fbabb4d0514a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R6bbe9b10be414440"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="2" r:id="R0a3b9d2ec5804e46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="Rcde75dc800f64967"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forwards" sheetId="4" r:id="R0518c2dc918f4c0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MoneyMarket" sheetId="5" r:id="R9b2941e80705460e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="6" r:id="Rc3eef09108a94324"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R82471ca4e16b417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R209c3f60f47c4b43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="9" r:id="R8ae8c72078424f6b"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="FC_AMT">'Inputs'!B2</x:definedName>
@@ -461,7 +461,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R17562561738f4e02"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc97e9f6fe46a4e8f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -845,7 +845,7 @@
         <x:v>S0_in</x:v>
       </x:c>
       <x:c r="B3" s="33" t="n">
-        <x:v>1.1</x:v>
+        <x:v>1.1535</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
         <x:v>USD per EUR</x:v>
@@ -856,7 +856,7 @@
         <x:v>F0_in</x:v>
       </x:c>
       <x:c r="B4" s="33" t="n">
-        <x:v>1.122</x:v>
+        <x:v>1.1738</x:v>
       </x:c>
       <x:c r="C4" s="10" t="str">
         <x:v>USD per EUR</x:v>
@@ -867,7 +867,7 @@
         <x:v>R_USD</x:v>
       </x:c>
       <x:c r="B5" s="34" t="n">
-        <x:v>0.035</x:v>
+        <x:v>0.0406</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
         <x:v>decimal (annual)</x:v>
@@ -878,7 +878,7 @@
         <x:v>R_FC</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>0.015</x:v>
+        <x:v>0.0225</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
         <x:v>decimal (annual)</x:v>
@@ -889,7 +889,7 @@
         <x:v>K_PUT</x:v>
       </x:c>
       <x:c r="B7" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>1.1535</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
         <x:v>USD per EUR</x:v>
@@ -900,7 +900,7 @@
         <x:v>K_CALL</x:v>
       </x:c>
       <x:c r="B8" s="33" t="n">
-        <x:v>1.2</x:v>
+        <x:v>1.1535</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
         <x:v>USD per EUR</x:v>
@@ -933,7 +933,7 @@
         <x:v>T_DAYS</x:v>
       </x:c>
       <x:c r="B11" s="32" t="n">
-        <x:v>365</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
         <x:v>days</x:v>
@@ -968,7 +968,7 @@
       </x:c>
       <x:c r="B3" s="39" t="n">
         <x:f>F0_in</x:f>
-        <x:v>1.122</x:v>
+        <x:v>1.1738</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -990,7 +990,7 @@
       </x:c>
       <x:c r="B6" s="42" t="n">
         <x:f>FC_AMT*F0_in</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1039,7 +1039,7 @@
       </x:c>
       <x:c r="B5" s="40" t="n">
         <x:f>FC_AMT/(1+R_FC*T_DAYS/360)</x:f>
-        <x:v>4432587.72829879</x:v>
+        <x:v>4401516.077760117</x:v>
       </x:c>
       <x:c r="C5" s="7"/>
     </x:row>
@@ -1070,7 +1070,7 @@
       </x:c>
       <x:c r="B9" s="40" t="n">
         <x:f>B5*S0_in</x:f>
-        <x:v>4875846.501128669</x:v>
+        <x:v>5077148.795696295</x:v>
       </x:c>
       <x:c r="C9" s="7"/>
     </x:row>
@@ -1101,7 +1101,7 @@
       </x:c>
       <x:c r="B13" s="42" t="n">
         <x:f>B9*(1+R_USD*T_DAYS/360)</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="C13" s="7"/>
     </x:row>
@@ -1140,7 +1140,7 @@
       </x:c>
       <x:c r="B4" s="40" t="n">
         <x:f>FC_AMT*MAX(S0_in,K_PUT)</x:f>
-        <x:v>4950000</x:v>
+        <x:v>5190750</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -1158,7 +1158,7 @@
       </x:c>
       <x:c r="B6" s="42" t="n">
         <x:f>B4-B5</x:f>
-        <x:v>4860000</x:v>
+        <x:v>5100750</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1186,7 +1186,7 @@
       </x:c>
       <x:c r="B10" s="42" t="n">
         <x:f>FC_AMT*S0_in-B9+FC_AMT*PREM_CALL</x:f>
-        <x:v>5040000</x:v>
+        <x:v>5280750</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1251,23 +1251,23 @@
       </x:c>
       <x:c r="B3" s="39" t="n">
         <x:f>ROUND(S0_in*(1+A3),3)</x:f>
-        <x:v>1.045</x:v>
+        <x:v>1.096</x:v>
       </x:c>
       <x:c r="C3" s="40" t="n">
         <x:f>FC_AMT*B3</x:f>
-        <x:v>4702500</x:v>
+        <x:v>4932000</x:v>
       </x:c>
       <x:c r="D3" s="40" t="n">
         <x:f>FORW_PROCEEDS</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
       <x:c r="E3" s="40" t="n">
         <x:f>MM_PROCEEDS</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="F3" s="40" t="n">
         <x:f>FC_AMT*MAX(B3,K_PUT)-FC_AMT*PREM_PUT</x:f>
-        <x:v>4612500</x:v>
+        <x:v>5100750</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -1276,23 +1276,23 @@
       </x:c>
       <x:c r="B4" s="39" t="n">
         <x:f>ROUND(S0_in*(1+A4),3)</x:f>
-        <x:v>1.056</x:v>
+        <x:v>1.107</x:v>
       </x:c>
       <x:c r="C4" s="40" t="n">
         <x:f>FC_AMT*B4</x:f>
-        <x:v>4752000</x:v>
+        <x:v>4981500</x:v>
       </x:c>
       <x:c r="D4" s="40" t="n">
         <x:f>FORW_PROCEEDS</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
       <x:c r="E4" s="40" t="n">
         <x:f>MM_PROCEEDS</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="F4" s="40" t="n">
         <x:f>FC_AMT*MAX(B4,K_PUT)-FC_AMT*PREM_PUT</x:f>
-        <x:v>4662000</x:v>
+        <x:v>5100750</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -1301,23 +1301,23 @@
       </x:c>
       <x:c r="B5" s="39" t="n">
         <x:f>ROUND(S0_in*(1+A5),3)</x:f>
-        <x:v>1.067</x:v>
+        <x:v>1.119</x:v>
       </x:c>
       <x:c r="C5" s="40" t="n">
         <x:f>FC_AMT*B5</x:f>
-        <x:v>4801500</x:v>
+        <x:v>5035500</x:v>
       </x:c>
       <x:c r="D5" s="40" t="n">
         <x:f>FORW_PROCEEDS</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
       <x:c r="E5" s="40" t="n">
         <x:f>MM_PROCEEDS</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="F5" s="40" t="n">
         <x:f>FC_AMT*MAX(B5,K_PUT)-FC_AMT*PREM_PUT</x:f>
-        <x:v>4711500</x:v>
+        <x:v>5100750</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1326,23 +1326,23 @@
       </x:c>
       <x:c r="B6" s="39" t="n">
         <x:f>ROUND(S0_in*(1+A6),3)</x:f>
-        <x:v>1.078</x:v>
+        <x:v>1.13</x:v>
       </x:c>
       <x:c r="C6" s="40" t="n">
         <x:f>FC_AMT*B6</x:f>
-        <x:v>4851000</x:v>
+        <x:v>5084999.999999999</x:v>
       </x:c>
       <x:c r="D6" s="40" t="n">
         <x:f>FORW_PROCEEDS</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
       <x:c r="E6" s="40" t="n">
         <x:f>MM_PROCEEDS</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="F6" s="40" t="n">
         <x:f>FC_AMT*MAX(B6,K_PUT)-FC_AMT*PREM_PUT</x:f>
-        <x:v>4761000</x:v>
+        <x:v>5100750</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1351,23 +1351,23 @@
       </x:c>
       <x:c r="B7" s="39" t="n">
         <x:f>ROUND(S0_in*(1+A7),3)</x:f>
-        <x:v>1.089</x:v>
+        <x:v>1.142</x:v>
       </x:c>
       <x:c r="C7" s="40" t="n">
         <x:f>FC_AMT*B7</x:f>
-        <x:v>4900500</x:v>
+        <x:v>5139000</x:v>
       </x:c>
       <x:c r="D7" s="40" t="n">
         <x:f>FORW_PROCEEDS</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
       <x:c r="E7" s="40" t="n">
         <x:f>MM_PROCEEDS</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="F7" s="40" t="n">
         <x:f>FC_AMT*MAX(B7,K_PUT)-FC_AMT*PREM_PUT</x:f>
-        <x:v>4810500</x:v>
+        <x:v>5100750</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1376,23 +1376,23 @@
       </x:c>
       <x:c r="B8" s="39" t="n">
         <x:f>ROUND(S0_in*(1+A8),3)</x:f>
-        <x:v>1.1</x:v>
+        <x:v>1.154</x:v>
       </x:c>
       <x:c r="C8" s="40" t="n">
         <x:f>FC_AMT*B8</x:f>
-        <x:v>4950000</x:v>
+        <x:v>5193000</x:v>
       </x:c>
       <x:c r="D8" s="40" t="n">
         <x:f>FORW_PROCEEDS</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
       <x:c r="E8" s="40" t="n">
         <x:f>MM_PROCEEDS</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="F8" s="40" t="n">
         <x:f>FC_AMT*MAX(B8,K_PUT)-FC_AMT*PREM_PUT</x:f>
-        <x:v>4860000</x:v>
+        <x:v>5103000</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1401,23 +1401,23 @@
       </x:c>
       <x:c r="B9" s="39" t="n">
         <x:f>ROUND(S0_in*(1+A9),3)</x:f>
-        <x:v>1.111</x:v>
+        <x:v>1.165</x:v>
       </x:c>
       <x:c r="C9" s="40" t="n">
         <x:f>FC_AMT*B9</x:f>
-        <x:v>4999500</x:v>
+        <x:v>5242500</x:v>
       </x:c>
       <x:c r="D9" s="40" t="n">
         <x:f>FORW_PROCEEDS</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
       <x:c r="E9" s="40" t="n">
         <x:f>MM_PROCEEDS</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="F9" s="40" t="n">
         <x:f>FC_AMT*MAX(B9,K_PUT)-FC_AMT*PREM_PUT</x:f>
-        <x:v>4909500</x:v>
+        <x:v>5152500</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1426,23 +1426,23 @@
       </x:c>
       <x:c r="B10" s="39" t="n">
         <x:f>ROUND(S0_in*(1+A10),3)</x:f>
-        <x:v>1.122</x:v>
+        <x:v>1.177</x:v>
       </x:c>
       <x:c r="C10" s="40" t="n">
         <x:f>FC_AMT*B10</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5296500</x:v>
       </x:c>
       <x:c r="D10" s="40" t="n">
         <x:f>FORW_PROCEEDS</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
       <x:c r="E10" s="40" t="n">
         <x:f>MM_PROCEEDS</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="F10" s="40" t="n">
         <x:f>FC_AMT*MAX(B10,K_PUT)-FC_AMT*PREM_PUT</x:f>
-        <x:v>4959000.000000001</x:v>
+        <x:v>5206500</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1451,23 +1451,23 @@
       </x:c>
       <x:c r="B11" s="39" t="n">
         <x:f>ROUND(S0_in*(1+A11),3)</x:f>
-        <x:v>1.133</x:v>
+        <x:v>1.188</x:v>
       </x:c>
       <x:c r="C11" s="40" t="n">
         <x:f>FC_AMT*B11</x:f>
-        <x:v>5098500</x:v>
+        <x:v>5346000</x:v>
       </x:c>
       <x:c r="D11" s="40" t="n">
         <x:f>FORW_PROCEEDS</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
       <x:c r="E11" s="40" t="n">
         <x:f>MM_PROCEEDS</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="F11" s="40" t="n">
         <x:f>FC_AMT*MAX(B11,K_PUT)-FC_AMT*PREM_PUT</x:f>
-        <x:v>5008500</x:v>
+        <x:v>5256000</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -1476,23 +1476,23 @@
       </x:c>
       <x:c r="B12" s="39" t="n">
         <x:f>ROUND(S0_in*(1+A12),3)</x:f>
-        <x:v>1.144</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="C12" s="40" t="n">
         <x:f>FC_AMT*B12</x:f>
-        <x:v>5148000</x:v>
+        <x:v>5400000</x:v>
       </x:c>
       <x:c r="D12" s="40" t="n">
         <x:f>FORW_PROCEEDS</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
       <x:c r="E12" s="40" t="n">
         <x:f>MM_PROCEEDS</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="F12" s="40" t="n">
         <x:f>FC_AMT*MAX(B12,K_PUT)-FC_AMT*PREM_PUT</x:f>
-        <x:v>5058000</x:v>
+        <x:v>5310000</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -1501,23 +1501,23 @@
       </x:c>
       <x:c r="B13" s="39" t="n">
         <x:f>ROUND(S0_in*(1+A13),3)</x:f>
-        <x:v>1.155</x:v>
+        <x:v>1.211</x:v>
       </x:c>
       <x:c r="C13" s="40" t="n">
         <x:f>FC_AMT*B13</x:f>
-        <x:v>5197500</x:v>
+        <x:v>5449500</x:v>
       </x:c>
       <x:c r="D13" s="40" t="n">
         <x:f>FORW_PROCEEDS</x:f>
-        <x:v>5049000.000000001</x:v>
+        <x:v>5282100</x:v>
       </x:c>
       <x:c r="E13" s="40" t="n">
         <x:f>MM_PROCEEDS</x:f>
-        <x:v>5048871.331828443</x:v>
+        <x:v>5282135.857684313</x:v>
       </x:c>
       <x:c r="F13" s="40" t="n">
         <x:f>FC_AMT*MAX(B13,K_PUT)-FC_AMT*PREM_PUT</x:f>
-        <x:v>5107500</x:v>
+        <x:v>5359500</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1525,7 +1525,7 @@
     <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R311c4c59063d4bdc"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d70a8a1028f4717"/>
 </x:worksheet>
 </file>
 
@@ -1563,7 +1563,7 @@
       </x:c>
       <x:c r="B4" s="39" t="n">
         <x:f>S0_in*(1+R_USD*T_DAYS/360)/(1+R_FC*T_DAYS/360)</x:f>
-        <x:v>1.1219714070729874</x:v>
+        <x:v>1.173807968374292</x:v>
       </x:c>
       <x:c r="C4" s="7"/>
     </x:row>
@@ -1573,7 +1573,7 @@
       </x:c>
       <x:c r="B5" s="39" t="n">
         <x:f>F0_in-B4</x:f>
-        <x:v>0.0000285929270127383</x:v>
+        <x:v>-0.000007968374291955627</x:v>
       </x:c>
       <x:c r="C5" s="7"/>
     </x:row>
@@ -1602,7 +1602,7 @@
       </x:c>
       <x:c r="B8" s="42" t="n">
         <x:f>FORW_PROCEEDS-MM_PROCEEDS</x:f>
-        <x:v>128.66817155759782</x:v>
+        <x:v>-35.85768431331962</x:v>
       </x:c>
       <x:c r="C8" s="7"/>
     </x:row>

</xml_diff>

<commit_message>
Align Stage 4 workbook documentation
</commit_message>
<xml_diff>
--- a/models/builds/2026-07-31-Ganoza-eur-receivable-hedge-model.xlsx
+++ b/models/builds/2026-07-31-Ganoza-eur-receivable-hedge-model.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R6bbe9b10be414440"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="2" r:id="R0a3b9d2ec5804e46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="Rcde75dc800f64967"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forwards" sheetId="4" r:id="R0518c2dc918f4c0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MoneyMarket" sheetId="5" r:id="R9b2941e80705460e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="6" r:id="Rc3eef09108a94324"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R82471ca4e16b417d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R209c3f60f47c4b43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="9" r:id="R8ae8c72078424f6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R9ebedb18324a4f6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="2" r:id="R85387585c7414486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="Rbb9372932a134c77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forwards" sheetId="4" r:id="R09083411d74b4a92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MoneyMarket" sheetId="5" r:id="Rea051bcb60ee432e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="6" r:id="R2ec4ce867bcd4017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" r:id="R4cad0262bdc549f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R76f10107703c47c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="9" r:id="R4afccdbb4cff4137"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="FC_AMT">'Inputs'!B2</x:definedName>
@@ -461,7 +461,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc97e9f6fe46a4e8f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc75d3c76485942e2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -694,7 +694,7 @@
         <x:v>Author:</x:v>
       </x:c>
       <x:c r="B4" s="10" t="str">
-        <x:v>Ethan Kainalu Ganoza</x:v>
+        <x:v>Ethan Ganoza</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -720,7 +720,7 @@
         <x:v>Spot Rate (S0_in):</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>ECB (placeholder)</x:v>
+        <x:v>ECB EUR/USD reference rate, 2026-08-07, 14:15 CET</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -728,7 +728,7 @@
         <x:v>Forward Rate (F0_in):</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>Parity-implied placeholder; dealer quote required in Stage 4</x:v>
+        <x:v>CIP-implied 1.1738 USD/EUR (not a dealer quote)</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -736,7 +736,7 @@
         <x:v>Interest Rates (R_USD, R_FC):</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>Fed H.15 / ECB (placeholder)</x:v>
+        <x:v>4.06% USD / 2.25% EUR (FRED / ECB proxies)</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -744,7 +744,7 @@
         <x:v>Option Premiums:</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Vendor TBD (placeholder)</x:v>
+        <x:v>0.0200 USD/EUR (scenario assumption)</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1525,7 +1525,7 @@
     <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d70a8a1028f4717"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96e5a3e377c5409a"/>
 </x:worksheet>
 </file>
 
@@ -1745,13 +1745,13 @@
         <x:v>Spot / EUR rate</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>ECB</x:v>
+        <x:v>ECB EUR/USD 1.1535 (2026-08-07)</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
-        <x:v>Placeholder</x:v>
+        <x:v>Populated</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
-        <x:v>Replace with as-of-date source</x:v>
+        <x:v>Reference rate, 14:15 CET</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1759,13 +1759,13 @@
         <x:v>USD / EUR interest rates</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>Fed H.15 / ECB</x:v>
+        <x:v>FRED DGS1 / ECB deposit facility</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
-        <x:v>Placeholder</x:v>
+        <x:v>Populated</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>Match date and ACT/360 convention</x:v>
+        <x:v>4.06% USD / 2.25% EUR rate proxies</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1773,13 +1773,13 @@
         <x:v>Forward rate</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>Dealer / market quote</x:v>
+        <x:v>CIP-implied forward</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
-        <x:v>Placeholder</x:v>
+        <x:v>Populated</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
-        <x:v>Compare to parity; document basis/spread</x:v>
+        <x:v>1.1738 USD/EUR; not a dealer quote</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1787,27 +1787,27 @@
         <x:v>Option premiums</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Vendor / OTC broker</x:v>
+        <x:v>Scenario assumption</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
-        <x:v>Placeholder</x:v>
+        <x:v>Documented</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>Record tenor, strike, and premium</x:v>
+        <x:v>0.0200 USD/EUR; retail quote not used</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A12" s="49" t="str">
-        <x:v>Put strike risk tolerance</x:v>
+        <x:v>Put strike decision</x:v>
       </x:c>
       <x:c r="B12" s="48" t="str">
-        <x:v>K_PUT = 1.00 protects a $4.41M net floor after premium</x:v>
+        <x:v>K_PUT = 1.1535 (at the money)</x:v>
       </x:c>
       <x:c r="C12" s="48" t="str">
-        <x:v>Decision required</x:v>
+        <x:v>Scenario convention</x:v>
       </x:c>
       <x:c r="D12" s="48" t="str">
-        <x:v>This accepts a $0.10/EUR decline from spot before the floor binds; set the strike based on the USD floor the business requires.</x:v>
+        <x:v>Net floor: 1.1335 USD/EUR / $5,100,750</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>